<commit_message>
Implementacion de if __name__ == "__main__": para evitar que el codigo se dispare
</commit_message>
<xml_diff>
--- a/datos/estadisticas.xlsx
+++ b/datos/estadisticas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,14 +446,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EDS Terpel Piedecuesta</t>
+          <t>CC la Florida</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>19.8</v>
+        <v>16.3</v>
       </c>
       <c r="D2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -464,14 +464,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Promotores del Oriente</t>
+          <t>CC Quinta Etapa</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>18.7</v>
+        <v>19.5</v>
       </c>
       <c r="D3" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -482,14 +482,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Promotores del Oriente</t>
+          <t>CC Cacique</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>13.2</v>
+        <v>17.7</v>
       </c>
       <c r="D4" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -500,14 +500,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>CC la Florida</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>18.9</v>
+        <v>19.3</v>
       </c>
       <c r="D5" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6">
@@ -518,14 +518,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EDS Terpel Piedecuesta</t>
+          <t>Éxito de la Rosita</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.7</v>
+        <v>16.8</v>
       </c>
       <c r="D6" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
@@ -540,10 +540,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>18.3</v>
+        <v>19.6</v>
       </c>
       <c r="D7" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
@@ -554,14 +554,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CC Cacique</t>
+          <t>CC Quinta Etapa</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.9</v>
+        <v>19.3</v>
       </c>
       <c r="D8" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9">
@@ -572,14 +572,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Promotores del Oriente</t>
+          <t>CC la Florida</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>17.9</v>
+        <v>16.4</v>
       </c>
       <c r="D9" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10">
@@ -590,14 +590,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Homecenter</t>
+          <t>EDS Terpel Piedecuesta</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>18.9</v>
+        <v>18.5</v>
       </c>
       <c r="D10" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11">
@@ -612,10 +612,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>18.3</v>
+        <v>17.5</v>
       </c>
       <c r="D11" t="n">
-        <v>136</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12">
@@ -630,10 +630,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18.1</v>
+        <v>19.7</v>
       </c>
       <c r="D12" t="n">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13">
@@ -644,14 +644,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.9</v>
+        <v>18.1</v>
       </c>
       <c r="D13" t="n">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14">
@@ -662,14 +662,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Éxito de la Rosita</t>
+          <t>CC Cacique</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>19.4</v>
+        <v>19.3</v>
       </c>
       <c r="D14" t="n">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>19.8</v>
+        <v>16.4</v>
       </c>
       <c r="D15" t="n">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16">
@@ -698,14 +698,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Éxito de la Rosita</t>
+          <t>EDS Terpel Piedecuesta</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="D16" t="n">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17">
@@ -716,50 +716,50 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Promotores del Oriente</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18.6</v>
+        <v>18.4</v>
       </c>
       <c r="D17" t="n">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BMW i4 eDrive40</t>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CC la Florida</t>
+          <t>Éxito de la Rosita</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="D18" t="n">
-        <v>262</v>
+        <v>252</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nissan LEAF Standard Range 52 kWh</t>
+          <t>BMW i4 eDrive40</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CC la Florida</t>
+          <t>Promotores del Oriente</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>19.6</v>
+        <v>19.2</v>
       </c>
       <c r="D19" t="n">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="20">
@@ -770,14 +770,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>CC Cacique</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.8</v>
+        <v>18.1</v>
       </c>
       <c r="D20" t="n">
-        <v>289</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21">
@@ -788,14 +788,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EDS Terpel Piedecuesta</t>
+          <t>Éxito de la Rosita</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>19.4</v>
+        <v>17.8</v>
       </c>
       <c r="D21" t="n">
-        <v>303</v>
+        <v>291</v>
       </c>
     </row>
     <row r="22">
@@ -806,14 +806,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CC Cacique</t>
+          <t>Promotores del Oriente</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18.9</v>
+        <v>19.1</v>
       </c>
       <c r="D22" t="n">
-        <v>315</v>
+        <v>297</v>
       </c>
     </row>
     <row r="23">
@@ -824,14 +824,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CC la Florida</t>
+          <t>EDS Terpel Piedecuesta</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>17.9</v>
+        <v>16.7</v>
       </c>
       <c r="D23" t="n">
-        <v>341</v>
+        <v>320</v>
       </c>
     </row>
     <row r="24">
@@ -842,14 +842,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>Éxito de la Rosita</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>18.6</v>
+        <v>19.4</v>
       </c>
       <c r="D24" t="n">
-        <v>345</v>
+        <v>326</v>
       </c>
     </row>
     <row r="25">
@@ -860,14 +860,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Promotores del Oriente</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>19.1</v>
+        <v>18.5</v>
       </c>
       <c r="D25" t="n">
-        <v>363</v>
+        <v>344</v>
       </c>
     </row>
     <row r="26">
@@ -878,14 +878,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="D26" t="n">
-        <v>381</v>
+        <v>368</v>
       </c>
     </row>
     <row r="27">
@@ -896,14 +896,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="D27" t="n">
-        <v>387</v>
+        <v>372</v>
       </c>
     </row>
     <row r="28">
@@ -914,14 +914,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Homecenter</t>
+          <t>EDS Terpel Piedecuesta</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>16.7</v>
       </c>
       <c r="D28" t="n">
-        <v>411</v>
+        <v>395</v>
       </c>
     </row>
     <row r="29">
@@ -932,14 +932,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>CC la Florida</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>19.6</v>
+        <v>19.2</v>
       </c>
       <c r="D29" t="n">
-        <v>417</v>
+        <v>405</v>
       </c>
     </row>
     <row r="30">
@@ -950,14 +950,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EDS Terpel Piedecuesta</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>15.3</v>
+        <v>19.2</v>
       </c>
       <c r="D30" t="n">
-        <v>440</v>
+        <v>421</v>
       </c>
     </row>
     <row r="31">
@@ -968,14 +968,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CC la Florida</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>19.5</v>
+        <v>19.2</v>
       </c>
       <c r="D31" t="n">
-        <v>455</v>
+        <v>443</v>
       </c>
     </row>
     <row r="32">
@@ -986,14 +986,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CC la Florida</t>
+          <t>CC Cacique</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.2</v>
+        <v>19.5</v>
       </c>
       <c r="D32" t="n">
-        <v>462</v>
+        <v>444</v>
       </c>
     </row>
     <row r="33">
@@ -1004,14 +1004,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EDS Terpel Piedecuesta</t>
+          <t>Promotores del Oriente</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>17</v>
+        <v>19.4</v>
       </c>
       <c r="D33" t="n">
-        <v>484</v>
+        <v>472</v>
       </c>
     </row>
     <row r="34">
@@ -1022,14 +1022,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CC Quinta Etapa</t>
+          <t>Homecenter</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>18.1</v>
+        <v>17.2</v>
       </c>
       <c r="D34" t="n">
-        <v>490</v>
+        <v>483</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D35" t="n">
+        <v>494</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implementacion de G=None, evita que corra la simulacion si no se ha cargado el grafo (Medida de seguridad extra)
</commit_message>
<xml_diff>
--- a/datos/estadisticas.xlsx
+++ b/datos/estadisticas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,14 +446,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Éxito de la Rosita</t>
+          <t>CC Cacique</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>19.5</v>
+        <v>19.3</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -464,14 +464,554 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CC la Florida</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D5" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CC Quinta Etapa</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>EDS Terpel Piedecuesta</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Promotores del Oriente</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>EDS Terpel Piedecuesta</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>16.9</v>
       </c>
-      <c r="D3" t="n">
-        <v>45</v>
+      <c r="D11" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CC la Florida</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="D12" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>EDS Terpel Piedecuesta</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>17</v>
+      </c>
+      <c r="D13" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>EDS Terpel Piedecuesta</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CC la Florida</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Promotores del Oriente</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EDS Terpel Piedecuesta</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CC Quinta Etapa</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CC la Florida</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D21" t="n">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CC Cacique</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>19</v>
+      </c>
+      <c r="D22" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D23" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Promotores del Oriente</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="D25" t="n">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D26" t="n">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CC la Florida</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D27" t="n">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>EDS Terpel Piedecuesta</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Homecenter</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D29" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Promotores del Oriente</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="D30" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Éxito de la Rosita</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="D31" t="n">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BMW i4 eDrive40</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CC Cacique</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D32" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nissan LEAF Standard Range 52 kWh</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>CC la Florida</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>20</v>
+      </c>
+      <c r="D33" t="n">
+        <v>490</v>
       </c>
     </row>
   </sheetData>

</xml_diff>